<commit_message>
📊 V9.2.1 daily run 2026-05-12_05:15
</commit_message>
<xml_diff>
--- a/paper_trades/dashboard_2026-05-12.xlsx
+++ b/paper_trades/dashboard_2026-05-12.xlsx
@@ -653,63 +653,63 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>14.64</v>
+        <v>15.01</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>13.88</v>
+        <v>14.23</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>15.34</v>
+        <v>15.74</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>15.89</v>
+        <v>16.31</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>11.78</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>53%</t>
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>14.51</v>
+        <v>14.68</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>-0.89</v>
+        <v>-2.2</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>0.89</v>
+        <v>1.27</v>
       </c>
       <c r="P4" s="8" t="n">
-        <v>-2.94</v>
+        <v>-3.06</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
@@ -720,22 +720,22 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -744,39 +744,39 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>15.01</v>
+        <v>12.24</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>14.23</v>
+        <v>11.61</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>15.74</v>
+        <v>13.07</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>16.31</v>
+        <v>13.7</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>11.78</v>
+        <v>16.08</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>53%</t>
+          <t>69%</t>
         </is>
       </c>
       <c r="L5" s="3" t="n">
         <v>2</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>14.68</v>
-      </c>
-      <c r="N5" s="7" t="n">
-        <v>-2.2</v>
+        <v>12.72</v>
+      </c>
+      <c r="N5" s="9" t="n">
+        <v>3.92</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>1.27</v>
+        <v>6.62</v>
       </c>
       <c r="P5" s="8" t="n">
-        <v>-3.06</v>
+        <v>-1.55</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -787,7 +787,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -797,12 +797,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -811,39 +811,39 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>12.24</v>
+        <v>25.85</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>11.61</v>
+        <v>24.88</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>13.07</v>
+        <v>26.72</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>13.7</v>
+        <v>27.41</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>16.08</v>
+        <v>14.35</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>69%</t>
+          <t>67%</t>
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>12.72</v>
-      </c>
-      <c r="N6" s="9" t="n">
-        <v>3.92</v>
+        <v>25.52</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>-1.28</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>6.62</v>
+        <v>0</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>-1.55</v>
+        <v>-1.97</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -864,12 +864,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -878,50 +878,50 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>25.85</v>
+        <v>90.63</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>24.88</v>
+        <v>86.5</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>26.72</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>27.41</v>
+        <v>97.36</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>14.35</v>
+        <v>14.18</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>25.52</v>
-      </c>
-      <c r="N7" s="7" t="n">
-        <v>-1.28</v>
+        <v>92.84999999999999</v>
+      </c>
+      <c r="N7" s="9" t="n">
+        <v>2.45</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>0</v>
+        <v>5.7</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>-1.97</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>🟢 Active</t>
+          <t>🟡 Partial</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -931,12 +931,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -945,36 +945,36 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>90.63</v>
+        <v>15.53</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>86.5</v>
+        <v>14.99</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>16.01</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>97.36</v>
+        <v>16.39</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>14.18</v>
+        <v>11.78</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>92.84999999999999</v>
+        <v>15.99</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>2.45</v>
+        <v>2.96</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>5.7</v>
+        <v>3.8</v>
       </c>
       <c r="P8" s="8" t="n">
         <v>0</v>
@@ -988,7 +988,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -998,12 +998,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1012,106 +1012,106 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>15.53</v>
+        <v>694.39</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>14.99</v>
+        <v>658.35</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>16.01</v>
+        <v>742</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>16.39</v>
+        <v>778.75</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>11.78</v>
+        <v>10.02</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>15.99</v>
+        <v>698.5</v>
       </c>
       <c r="N9" s="9" t="n">
-        <v>2.96</v>
+        <v>0.59</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>3.8</v>
+        <v>2.54</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>0</v>
+        <v>-0.34</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>🟡 Partial</t>
+          <t>🟢 Active</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>694.39</v>
+        <v>28.9</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>658.35</v>
+        <v>27.4</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>742</v>
+        <v>30.89</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>778.75</v>
+        <v>32.42</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>10.02</v>
+        <v>12.9</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="L10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>698.5</v>
-      </c>
-      <c r="N10" s="9" t="n">
-        <v>0.59</v>
+        <v>28.84</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>-0.21</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>2.54</v>
+        <v>0</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>-0.34</v>
+        <v>-4.36</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1122,7 +1122,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0020</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1132,12 +1132,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1146,30 +1146,30 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>32.56</v>
+        <v>45.31</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>30.88</v>
+        <v>43.36</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>34.52</v>
+        <v>47.08</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>36.04</v>
+        <v>48.47</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>15.98</v>
+        <v>12.93</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>76%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="L11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>32.56</v>
+        <v>45.31</v>
       </c>
       <c r="N11" s="8" t="n">
         <v>0</v>
@@ -1189,7 +1189,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0021</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1199,12 +1199,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1213,30 +1213,30 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>45.31</v>
+        <v>32.56</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>43.36</v>
+        <v>30.88</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>47.08</v>
+        <v>34.52</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>48.47</v>
+        <v>36.04</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>13.05</v>
+        <v>12.53</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>76%</t>
         </is>
       </c>
       <c r="L12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>45.31</v>
+        <v>32.56</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>0</v>
@@ -1256,7 +1256,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0022</t>
+          <t>T0025</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1266,44 +1266,44 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>28.9</v>
+        <v>100.3</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>27.4</v>
+        <v>95.5</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>30.89</v>
+        <v>104.7</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>32.42</v>
+        <v>108.16</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>12.9</v>
+        <v>9.9</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="L13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>28.9</v>
+        <v>100.3</v>
       </c>
       <c r="N13" s="8" t="n">
         <v>0</v>
@@ -1334,7 +1334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1631,7 +1631,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1641,39 +1641,39 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>43.19</v>
+        <v>14.64</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>43.88</v>
+        <v>14.51</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J7" s="9" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>7</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>-0.0089</v>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
@@ -1682,42 +1682,42 @@
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.0188</v>
+        <v>0.0089</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0294</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>32.16</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>13</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -1726,64 +1726,64 @@
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>137.37</v>
+        <v>32.56</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>143</v>
+        <v>30.73</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J8" s="9" t="n">
-        <v>0.04099999999999999</v>
-      </c>
-      <c r="K8" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>1</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>-0.0563</v>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0.0432</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0608</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>30.86</v>
+        <v>15.98</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>22.9</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1792,44 +1792,44 @@
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>27.31</v>
+        <v>45.31</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>27.86</v>
+        <v>43.14</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J9" s="9" t="n">
-        <v>0.0201</v>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>1</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>-0.0478</v>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0.0392</v>
+        <v>0</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.0925</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>26.27</v>
+        <v>13.05</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>23.9</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1858,16 +1858,16 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>37.25</v>
+        <v>43.19</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>38.14</v>
+        <v>43.88</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>0.0239</v>
+        <v>0.016</v>
       </c>
       <c r="K10" s="11" t="inlineStr">
         <is>
@@ -1880,22 +1880,22 @@
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0188</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.0016</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>23.8</v>
+        <v>32.16</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>27.9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1910,12 +1910,12 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1924,20 +1924,20 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>105.01</v>
+        <v>137.37</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>105</v>
+        <v>143</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J11" s="7" t="n">
-        <v>-0.0001</v>
-      </c>
-      <c r="K11" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+      <c r="J11" s="9" t="n">
+        <v>0.04099999999999999</v>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -1946,22 +1946,22 @@
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0432</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.002</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>10.01</v>
+        <v>30.86</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>17.6</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1971,39 +1971,39 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>26.25</v>
+        <v>27.31</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>25.64</v>
+        <v>27.86</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>-0.0232</v>
-      </c>
-      <c r="K12" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>0.0201</v>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
@@ -2012,22 +2012,22 @@
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0392</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0114</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>16.26</v>
+        <v>26.27</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>31.4</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2037,35 +2037,35 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>10.7</v>
+        <v>37.25</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>10.73</v>
+        <v>38.14</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>0.0028</v>
+        <v>0.0239</v>
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
@@ -2078,22 +2078,22 @@
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0379</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>12.8</v>
+        <v>23.8</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>14.8</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2103,122 +2103,320 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>11.92</v>
+        <v>105.01</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>11.24</v>
+        <v>105</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>-0.0568</v>
+        <v>-0.0001</v>
       </c>
       <c r="K14" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0</v>
+        <v>0.0075</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.022</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>12</v>
+        <v>10.01</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>33.5</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
+          <t>T0005</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>4145</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>صناعية</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M15" s="8" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="N15" s="8" t="n">
+        <v>-0.0316</v>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>16.26</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J16" s="9" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M16" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N16" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O16" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P16" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M17" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O17" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P17" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G18" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H15" s="5" t="n">
+      <c r="H18" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I15" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" s="7" t="n">
+      <c r="I18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="7" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K15" s="10" t="inlineStr">
+      <c r="K18" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="L18" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M15" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="8" t="n">
+      <c r="M18" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O15" s="6" t="n">
+      <c r="O18" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P15" s="6" t="n">
+      <c r="P18" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -2236,7 +2434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2253,7 +2451,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-12T02:02:25</t>
+          <t>محسوب في: 2026-05-12T05:15:09</t>
         </is>
       </c>
     </row>
@@ -2277,7 +2475,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -2307,7 +2505,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -2318,7 +2516,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>40.0%</t>
         </is>
       </c>
     </row>
@@ -2342,7 +2540,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.38%</t>
+          <t>-3.51%</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2551,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.95</v>
+        <v>0.61</v>
       </c>
     </row>
     <row r="13">
@@ -2364,7 +2562,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-0.99%</t>
+          <t>-12.29%</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2650,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C25" s="3" t="n">
         <v>0</v>
@@ -2464,7 +2662,7 @@
       </c>
       <c r="E25" s="17" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-4.08%</t>
         </is>
       </c>
     </row>
@@ -2498,19 +2696,19 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D27" s="16" t="inlineStr">
-        <is>
-          <t>71.4%</t>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>55.6%</t>
         </is>
       </c>
       <c r="E27" s="16" t="inlineStr">
         <is>
-          <t>+2.39%</t>
+          <t>+0.70%</t>
         </is>
       </c>
     </row>
@@ -2581,7 +2779,7 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C34" s="3" t="n">
         <v>0</v>
@@ -2593,7 +2791,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>-3.31%</t>
+          <t>-4.09%</t>
         </is>
       </c>
     </row>
@@ -2650,19 +2848,19 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C37" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>50.0%</t>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>33.3%</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>-2.04%</t>
+          <t>-2.95%</t>
         </is>
       </c>
     </row>
@@ -2712,18 +2910,41 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>تجزئة</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>-0.89%</t>
+        </is>
+      </c>
+    </row>
     <row r="41"/>
-    <row r="42">
-      <c r="A42" s="24" t="inlineStr">
+    <row r="42"/>
+    <row r="43">
+      <c r="A43" s="24" t="inlineStr">
         <is>
           <t>⚠️ الأسهم المُتعِبة (Win Rate &lt; 30% مع 3+ صفقات)</t>
         </is>
       </c>
     </row>
-    <row r="43"/>
-    <row r="44">
-      <c r="A44" s="25" t="inlineStr">
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" s="25" t="inlineStr">
         <is>
           <t>(لا توجد بعد - يحتاج 3+ صفقات لكل سهم)</t>
         </is>
@@ -2744,7 +2965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3298,6 +3519,129 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>4020</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>تجزئة</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>-0.89%</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>-0.89%</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>-0.89%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>2370</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>-5.63%</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>-5.63%</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>-5.63%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>2280</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>زراعة وأغذية</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>-4.78%</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>-4.78%</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>-4.78%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-12_05:31
</commit_message>
<xml_diff>
--- a/paper_trades/dashboard_2026-05-12.xlsx
+++ b/paper_trades/dashboard_2026-05-12.xlsx
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M4" s="5" t="n">
         <v>14.68</v>
@@ -764,7 +764,7 @@
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M5" s="5" t="n">
         <v>12.72</v>
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M6" s="5" t="n">
         <v>25.52</v>
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M7" s="5" t="n">
         <v>92.84999999999999</v>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M8" s="5" t="n">
         <v>15.99</v>
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="5" t="n">
         <v>698.5</v>
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" s="5" t="n">
         <v>28.84</v>
@@ -1122,7 +1122,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0023</t>
+          <t>T0025</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1132,12 +1132,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1146,39 +1146,39 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>45.31</v>
+        <v>100.3</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>43.36</v>
+        <v>95.5</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>47.08</v>
+        <v>104.7</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>48.47</v>
+        <v>108.16</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>12.93</v>
+        <v>9.9</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="L11" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>45.31</v>
-      </c>
-      <c r="N11" s="8" t="n">
-        <v>0</v>
+        <v>100.1</v>
+      </c>
+      <c r="N11" s="7" t="n">
+        <v>-0.2</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="P11" s="8" t="n">
-        <v>0</v>
+        <v>-2.49</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
@@ -1189,7 +1189,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0024</t>
+          <t>T0026</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1199,12 +1199,12 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1213,30 +1213,30 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>32.56</v>
+        <v>45.31</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>30.88</v>
+        <v>43.36</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>34.52</v>
+        <v>47.08</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>36.04</v>
+        <v>48.47</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>12.53</v>
+        <v>12.84</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>76%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="L12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>32.56</v>
+        <v>45.31</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>0</v>
@@ -1256,7 +1256,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0025</t>
+          <t>T0027</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -1266,12 +1266,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>7040</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>اتصالات</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1280,30 +1280,30 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>100.3</v>
+        <v>32.56</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>95.5</v>
+        <v>30.88</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>104.7</v>
+        <v>34.52</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>108.16</v>
+        <v>36.04</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>9.9</v>
+        <v>12.52</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>76%</t>
         </is>
       </c>
       <c r="L13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>100.3</v>
+        <v>32.56</v>
       </c>
       <c r="N13" s="8" t="n">
         <v>0</v>
@@ -1334,7 +1334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1829,22 +1829,22 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1858,64 +1858,64 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>43.19</v>
+        <v>45.31</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>43.88</v>
+        <v>43.14</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J10" s="9" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>1</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>-0.0478</v>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0.0188</v>
+        <v>0</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0925</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>32.16</v>
+        <v>12.93</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>13</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1924,44 +1924,44 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>137.37</v>
+        <v>32.56</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>143</v>
+        <v>30.73</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J11" s="9" t="n">
-        <v>0.04099999999999999</v>
-      </c>
-      <c r="K11" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>1</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>-0.0563</v>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0.0432</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0608</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>30.86</v>
+        <v>12.53</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>22.9</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1976,12 +1976,12 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1990,16 +1990,16 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>27.31</v>
+        <v>43.19</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>27.86</v>
+        <v>43.88</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.0201</v>
+        <v>0.016</v>
       </c>
       <c r="K12" s="11" t="inlineStr">
         <is>
@@ -2012,22 +2012,22 @@
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0.0392</v>
+        <v>0.0188</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.0016</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>26.27</v>
+        <v>32.16</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>23.9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2042,12 +2042,12 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -2056,16 +2056,16 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>37.25</v>
+        <v>137.37</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>38.14</v>
+        <v>143</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>0.0239</v>
+        <v>0.04099999999999999</v>
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
@@ -2078,22 +2078,22 @@
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0432</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.002</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>23.8</v>
+        <v>30.86</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>27.9</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2108,12 +2108,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -2122,20 +2122,20 @@
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>105.01</v>
+        <v>27.31</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>105</v>
+        <v>27.86</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J14" s="7" t="n">
-        <v>-0.0001</v>
-      </c>
-      <c r="K14" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+      <c r="J14" s="9" t="n">
+        <v>0.0201</v>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
@@ -2144,22 +2144,22 @@
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0392</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.0114</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>10.01</v>
+        <v>26.27</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>17.6</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2169,39 +2169,39 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>26.25</v>
+        <v>37.25</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>25.64</v>
+        <v>38.14</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>-0.0232</v>
-      </c>
-      <c r="K15" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>0.0239</v>
+      </c>
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -2210,22 +2210,22 @@
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0379</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0212</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>16.26</v>
+        <v>23.8</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>31.4</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2235,39 +2235,39 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>10.7</v>
+        <v>105.01</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>10.73</v>
+        <v>105</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J16" s="9" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K16" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>5</v>
+      </c>
+      <c r="J16" s="7" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="K16" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -2276,22 +2276,22 @@
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0075</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.022</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>12.8</v>
+        <v>10.01</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>14.8</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0005</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -2301,122 +2301,254 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>11.92</v>
+        <v>26.25</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>11.24</v>
+        <v>25.64</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>-0.0568</v>
+        <v>-0.0232</v>
       </c>
       <c r="K17" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M17" s="8" t="n">
-        <v>0</v>
+        <v>0.0011</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.0316</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>12</v>
+        <v>16.26</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>33.5</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J18" s="9" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M18" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N18" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O18" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P18" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O19" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P19" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G18" s="5" t="n">
+      <c r="G20" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H18" s="5" t="n">
+      <c r="H20" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I18" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="7" t="n">
+      <c r="I20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="7" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K18" s="10" t="inlineStr">
+      <c r="K20" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr">
+      <c r="L20" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M18" s="8" t="n">
+      <c r="M20" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N18" s="8" t="n">
+      <c r="N20" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O18" s="6" t="n">
+      <c r="O20" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P18" s="6" t="n">
+      <c r="P20" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -2451,7 +2583,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-12T05:15:09</t>
+          <t>محسوب في: 2026-05-12T05:31:52</t>
         </is>
       </c>
     </row>
@@ -2475,7 +2607,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -2505,7 +2637,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
@@ -2516,7 +2648,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>40.0%</t>
+          <t>35.3%</t>
         </is>
       </c>
     </row>
@@ -2540,7 +2672,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.51%</t>
+          <t>-3.82%</t>
         </is>
       </c>
     </row>
@@ -2551,7 +2683,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.61</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="13">
@@ -2562,7 +2694,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-12.29%</t>
+          <t>-22.7%</t>
         </is>
       </c>
     </row>
@@ -2696,19 +2828,19 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>55.6%</t>
-        </is>
-      </c>
-      <c r="E27" s="16" t="inlineStr">
-        <is>
-          <t>+0.70%</t>
+          <t>45.5%</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>-0.37%</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2911,7 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C34" s="3" t="n">
         <v>0</v>
@@ -2791,7 +2923,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>-4.09%</t>
+          <t>-4.47%</t>
         </is>
       </c>
     </row>
@@ -2848,19 +2980,19 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C37" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D37" s="17" t="inlineStr">
         <is>
-          <t>33.3%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>-2.95%</t>
+          <t>-3.41%</t>
         </is>
       </c>
     </row>
@@ -3572,13 +3704,13 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
@@ -3613,13 +3745,13 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>

</xml_diff>